<commit_message>
Cap nhat sua mau 08-TCCB
</commit_message>
<xml_diff>
--- a/QLNS/FileExcels/BC_MangLuoiLD_08_TCCB.xlsx
+++ b/QLNS/FileExcels/BC_MangLuoiLD_08_TCCB.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="64">
   <si>
     <t>NGÂN HÀNG CHÍNH SÁCH XÃ HỘI</t>
   </si>
@@ -186,9 +186,6 @@
     <t>%SoToTKVVBQ_CanBo</t>
   </si>
   <si>
-    <t>Tỷ lệ Nợ quá hạn (%)</t>
-  </si>
-  <si>
     <t>Tỷ lệ thu lãi (%)</t>
   </si>
   <si>
@@ -198,10 +195,22 @@
     <t>17</t>
   </si>
   <si>
-    <t>%TyLeNQH</t>
-  </si>
-  <si>
     <t>%TyLeThuLai</t>
+  </si>
+  <si>
+    <t>%TyLeNQHNKH</t>
+  </si>
+  <si>
+    <t>Tỷ lệ Nợ quá hạn (bao gồm NQH + Nợ khoanh) (%)</t>
+  </si>
+  <si>
+    <t>Chênh lệch Thu - Chi  (chưa có lương, không tính chi phí trả lãi huy động vốn tiền gửi) (Triệu đồng)</t>
+  </si>
+  <si>
+    <t>%ChenhLechThuChi</t>
+  </si>
+  <si>
+    <t>18</t>
   </si>
 </sst>
 </file>
@@ -409,8 +418,8 @@
     <xf numFmtId="4" fontId="6" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="6" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="4" fontId="6" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -448,8 +457,8 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="4" fontId="6" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    <xf numFmtId="3" fontId="6" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -756,7 +765,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:R10"/>
+  <dimension ref="A1:S10"/>
   <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.88671875" style="1" customWidth="1"/>
@@ -771,19 +780,20 @@
     <col min="12" max="12" width="8.88671875" style="2" customWidth="1"/>
     <col min="13" max="13" width="8.5546875" style="2" customWidth="1"/>
     <col min="14" max="15" width="8.21875" style="2" customWidth="1"/>
-    <col min="16" max="16" width="6.33203125" style="2" customWidth="1"/>
-    <col min="17" max="17" width="7" style="2" customWidth="1"/>
-    <col min="18" max="18" width="13.5546875" style="2" customWidth="1"/>
-    <col min="19" max="16384" width="9.109375" style="2"/>
+    <col min="16" max="16" width="8.33203125" style="2" customWidth="1"/>
+    <col min="17" max="17" width="6.88671875" style="2" customWidth="1"/>
+    <col min="18" max="18" width="12.5546875" style="2" customWidth="1"/>
+    <col min="19" max="19" width="13.5546875" style="2" customWidth="1"/>
+    <col min="20" max="16384" width="9.109375" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="Q1" s="1"/>
-      <c r="R1" s="3" t="s">
+    <row r="1" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="R1" s="1"/>
+      <c r="S1" s="3" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="2" spans="1:18" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="23" t="s">
         <v>0</v>
       </c>
@@ -805,8 +815,9 @@
       <c r="P2" s="23"/>
       <c r="Q2" s="23"/>
       <c r="R2" s="23"/>
+      <c r="S2" s="23"/>
     </row>
-    <row r="3" spans="1:18" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:19" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="23" t="s">
         <v>22</v>
       </c>
@@ -828,8 +839,9 @@
       <c r="P3" s="24"/>
       <c r="Q3" s="24"/>
       <c r="R3" s="24"/>
+      <c r="S3" s="24"/>
     </row>
-    <row r="4" spans="1:18" ht="23.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:19" ht="23.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="23" t="s">
         <v>48</v>
       </c>
@@ -850,8 +862,9 @@
       <c r="P4" s="23"/>
       <c r="Q4" s="23"/>
       <c r="R4" s="23"/>
+      <c r="S4" s="23"/>
     </row>
-    <row r="5" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="23" t="s">
         <v>4</v>
       </c>
@@ -872,9 +885,10 @@
       <c r="P5" s="23"/>
       <c r="Q5" s="23"/>
       <c r="R5" s="23"/>
+      <c r="S5" s="23"/>
     </row>
-    <row r="6" spans="1:18" ht="3" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="7" spans="1:18" s="4" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:19" ht="3" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="7" spans="1:19" s="4" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="13" t="s">
         <v>3</v>
       </c>
@@ -921,16 +935,19 @@
         <v>47</v>
       </c>
       <c r="P7" s="15" t="s">
+        <v>60</v>
+      </c>
+      <c r="Q7" s="17" t="s">
         <v>55</v>
       </c>
-      <c r="Q7" s="17" t="s">
-        <v>56</v>
-      </c>
-      <c r="R7" s="15" t="s">
+      <c r="R7" s="17" t="s">
+        <v>61</v>
+      </c>
+      <c r="S7" s="15" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="8" spans="1:18" s="4" customFormat="1" ht="69" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:19" s="4" customFormat="1" ht="84" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="14"/>
       <c r="B8" s="14"/>
       <c r="C8" s="21"/>
@@ -948,9 +965,10 @@
       <c r="O8" s="18"/>
       <c r="P8" s="16"/>
       <c r="Q8" s="18"/>
-      <c r="R8" s="16"/>
+      <c r="R8" s="18"/>
+      <c r="S8" s="16"/>
     </row>
-    <row r="9" spans="1:18" s="9" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:19" s="9" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="8" t="s">
         <v>25</v>
       </c>
@@ -1000,13 +1018,16 @@
         <v>40</v>
       </c>
       <c r="Q9" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="R9" s="8" t="s">
         <v>57</v>
       </c>
-      <c r="R9" s="8" t="s">
-        <v>58</v>
+      <c r="S9" s="8" t="s">
+        <v>63</v>
       </c>
     </row>
-    <row r="10" spans="1:18" s="4" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:19" s="4" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="5" t="s">
         <v>12</v>
       </c>
@@ -1049,25 +1070,28 @@
       <c r="N10" s="11" t="s">
         <v>54</v>
       </c>
-      <c r="O10" s="12" t="s">
+      <c r="O10" s="25" t="s">
         <v>50</v>
       </c>
       <c r="P10" s="11" t="s">
         <v>59</v>
       </c>
-      <c r="Q10" s="25" t="s">
-        <v>60</v>
-      </c>
-      <c r="R10" s="10" t="s">
+      <c r="Q10" s="12" t="s">
+        <v>58</v>
+      </c>
+      <c r="R10" s="12" t="s">
+        <v>62</v>
+      </c>
+      <c r="S10" s="10" t="s">
         <v>24</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="24">
-    <mergeCell ref="F2:R2"/>
-    <mergeCell ref="F3:R3"/>
-    <mergeCell ref="A4:R4"/>
-    <mergeCell ref="A5:R5"/>
+  <mergeCells count="25">
+    <mergeCell ref="F2:S2"/>
+    <mergeCell ref="F3:S3"/>
+    <mergeCell ref="A4:S4"/>
+    <mergeCell ref="A5:S5"/>
     <mergeCell ref="A2:D2"/>
     <mergeCell ref="A3:D3"/>
     <mergeCell ref="A7:A8"/>
@@ -1079,8 +1103,8 @@
     <mergeCell ref="F7:F8"/>
     <mergeCell ref="G7:G8"/>
     <mergeCell ref="I7:I8"/>
+    <mergeCell ref="S7:S8"/>
     <mergeCell ref="R7:R8"/>
-    <mergeCell ref="Q7:Q8"/>
     <mergeCell ref="J7:J8"/>
     <mergeCell ref="L7:L8"/>
     <mergeCell ref="M7:M8"/>
@@ -1088,9 +1112,10 @@
     <mergeCell ref="N7:N8"/>
     <mergeCell ref="O7:O8"/>
     <mergeCell ref="P7:P8"/>
+    <mergeCell ref="Q7:Q8"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.6" right="0.5" top="0.6" bottom="0.5" header="0.05" footer="0.05"/>
-  <pageSetup paperSize="9" scale="80" orientation="landscape" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="70" orientation="landscape" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Cap nhat 08 và ngay HL quyet dinh 30 ngày
</commit_message>
<xml_diff>
--- a/QLNS/FileExcels/BC_MangLuoiLD_08_TCCB.xlsx
+++ b/QLNS/FileExcels/BC_MangLuoiLD_08_TCCB.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="66">
   <si>
     <t>NGÂN HÀNG CHÍNH SÁCH XÃ HỘI</t>
   </si>
@@ -211,6 +211,12 @@
   </si>
   <si>
     <t>18</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mã đơn vị </t>
+  </si>
+  <si>
+    <t>%DonVi_Cd</t>
   </si>
 </sst>
 </file>
@@ -421,6 +427,9 @@
     <xf numFmtId="4" fontId="6" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="3" fontId="6" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -456,9 +465,6 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="6" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -765,354 +771,368 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:S10"/>
+  <dimension ref="A1:T10"/>
   <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="4.88671875" style="1" customWidth="1"/>
-    <col min="2" max="2" width="22.21875" style="2" customWidth="1"/>
-    <col min="3" max="4" width="7.33203125" style="2" customWidth="1"/>
-    <col min="5" max="5" width="11.33203125" style="2" customWidth="1"/>
-    <col min="6" max="6" width="9.33203125" style="2" customWidth="1"/>
-    <col min="7" max="8" width="7.33203125" style="2" customWidth="1"/>
-    <col min="9" max="9" width="7.77734375" style="2" customWidth="1"/>
-    <col min="10" max="10" width="11.33203125" style="2" customWidth="1"/>
-    <col min="11" max="11" width="9.5546875" style="2" customWidth="1"/>
-    <col min="12" max="12" width="8.88671875" style="2" customWidth="1"/>
-    <col min="13" max="13" width="8.5546875" style="2" customWidth="1"/>
-    <col min="14" max="15" width="8.21875" style="2" customWidth="1"/>
-    <col min="16" max="16" width="8.33203125" style="2" customWidth="1"/>
-    <col min="17" max="17" width="6.88671875" style="2" customWidth="1"/>
-    <col min="18" max="18" width="12.5546875" style="2" customWidth="1"/>
-    <col min="19" max="19" width="13.5546875" style="2" customWidth="1"/>
-    <col min="20" max="16384" width="9.109375" style="2"/>
+    <col min="1" max="1" width="3.77734375" style="1" customWidth="1"/>
+    <col min="2" max="2" width="7" style="1" customWidth="1"/>
+    <col min="3" max="3" width="22.21875" style="2" customWidth="1"/>
+    <col min="4" max="5" width="7.33203125" style="2" customWidth="1"/>
+    <col min="6" max="6" width="11.33203125" style="2" customWidth="1"/>
+    <col min="7" max="7" width="9.33203125" style="2" customWidth="1"/>
+    <col min="8" max="9" width="7.33203125" style="2" customWidth="1"/>
+    <col min="10" max="10" width="7.77734375" style="2" customWidth="1"/>
+    <col min="11" max="11" width="11.33203125" style="2" customWidth="1"/>
+    <col min="12" max="12" width="9.5546875" style="2" customWidth="1"/>
+    <col min="13" max="13" width="8.88671875" style="2" customWidth="1"/>
+    <col min="14" max="14" width="8.5546875" style="2" customWidth="1"/>
+    <col min="15" max="16" width="8.21875" style="2" customWidth="1"/>
+    <col min="17" max="17" width="8.33203125" style="2" customWidth="1"/>
+    <col min="18" max="18" width="6.88671875" style="2" customWidth="1"/>
+    <col min="19" max="19" width="12.5546875" style="2" customWidth="1"/>
+    <col min="20" max="20" width="13.5546875" style="2" customWidth="1"/>
+    <col min="21" max="16384" width="9.109375" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="R1" s="1"/>
-      <c r="S1" s="3" t="s">
+    <row r="1" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="S1" s="1"/>
+      <c r="T1" s="3" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="2" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="23" t="s">
+    <row r="2" spans="1:20" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="24" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="23"/>
-      <c r="C2" s="23"/>
-      <c r="D2" s="23"/>
-      <c r="F2" s="23" t="s">
+      <c r="B2" s="24"/>
+      <c r="C2" s="24"/>
+      <c r="D2" s="24"/>
+      <c r="E2" s="24"/>
+      <c r="G2" s="24" t="s">
         <v>1</v>
       </c>
-      <c r="G2" s="23"/>
-      <c r="H2" s="23"/>
-      <c r="I2" s="23"/>
-      <c r="J2" s="23"/>
-      <c r="K2" s="23"/>
-      <c r="L2" s="23"/>
-      <c r="M2" s="23"/>
-      <c r="N2" s="23"/>
-      <c r="O2" s="23"/>
-      <c r="P2" s="23"/>
-      <c r="Q2" s="23"/>
-      <c r="R2" s="23"/>
-      <c r="S2" s="23"/>
+      <c r="H2" s="24"/>
+      <c r="I2" s="24"/>
+      <c r="J2" s="24"/>
+      <c r="K2" s="24"/>
+      <c r="L2" s="24"/>
+      <c r="M2" s="24"/>
+      <c r="N2" s="24"/>
+      <c r="O2" s="24"/>
+      <c r="P2" s="24"/>
+      <c r="Q2" s="24"/>
+      <c r="R2" s="24"/>
+      <c r="S2" s="24"/>
+      <c r="T2" s="24"/>
     </row>
-    <row r="3" spans="1:19" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="23" t="s">
+    <row r="3" spans="1:20" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="24" t="s">
         <v>22</v>
       </c>
-      <c r="B3" s="23"/>
-      <c r="C3" s="23"/>
-      <c r="D3" s="23"/>
-      <c r="F3" s="24" t="s">
+      <c r="B3" s="24"/>
+      <c r="C3" s="24"/>
+      <c r="D3" s="24"/>
+      <c r="E3" s="24"/>
+      <c r="G3" s="25" t="s">
         <v>2</v>
       </c>
-      <c r="G3" s="24"/>
-      <c r="H3" s="24"/>
-      <c r="I3" s="24"/>
-      <c r="J3" s="24"/>
-      <c r="K3" s="24"/>
-      <c r="L3" s="24"/>
-      <c r="M3" s="24"/>
-      <c r="N3" s="24"/>
-      <c r="O3" s="24"/>
-      <c r="P3" s="24"/>
-      <c r="Q3" s="24"/>
-      <c r="R3" s="24"/>
-      <c r="S3" s="24"/>
+      <c r="H3" s="25"/>
+      <c r="I3" s="25"/>
+      <c r="J3" s="25"/>
+      <c r="K3" s="25"/>
+      <c r="L3" s="25"/>
+      <c r="M3" s="25"/>
+      <c r="N3" s="25"/>
+      <c r="O3" s="25"/>
+      <c r="P3" s="25"/>
+      <c r="Q3" s="25"/>
+      <c r="R3" s="25"/>
+      <c r="S3" s="25"/>
+      <c r="T3" s="25"/>
     </row>
-    <row r="4" spans="1:19" ht="23.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="23" t="s">
+    <row r="4" spans="1:20" ht="23.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="24" t="s">
         <v>48</v>
       </c>
-      <c r="B4" s="23"/>
-      <c r="C4" s="23"/>
-      <c r="D4" s="23"/>
-      <c r="E4" s="23"/>
-      <c r="F4" s="23"/>
-      <c r="G4" s="23"/>
-      <c r="H4" s="23"/>
-      <c r="I4" s="23"/>
-      <c r="J4" s="23"/>
-      <c r="K4" s="23"/>
-      <c r="L4" s="23"/>
-      <c r="M4" s="23"/>
-      <c r="N4" s="23"/>
-      <c r="O4" s="23"/>
-      <c r="P4" s="23"/>
-      <c r="Q4" s="23"/>
-      <c r="R4" s="23"/>
-      <c r="S4" s="23"/>
+      <c r="B4" s="24"/>
+      <c r="C4" s="24"/>
+      <c r="D4" s="24"/>
+      <c r="E4" s="24"/>
+      <c r="F4" s="24"/>
+      <c r="G4" s="24"/>
+      <c r="H4" s="24"/>
+      <c r="I4" s="24"/>
+      <c r="J4" s="24"/>
+      <c r="K4" s="24"/>
+      <c r="L4" s="24"/>
+      <c r="M4" s="24"/>
+      <c r="N4" s="24"/>
+      <c r="O4" s="24"/>
+      <c r="P4" s="24"/>
+      <c r="Q4" s="24"/>
+      <c r="R4" s="24"/>
+      <c r="S4" s="24"/>
+      <c r="T4" s="24"/>
     </row>
-    <row r="5" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="23" t="s">
+    <row r="5" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="24" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="23"/>
-      <c r="C5" s="23"/>
-      <c r="D5" s="23"/>
-      <c r="E5" s="23"/>
-      <c r="F5" s="23"/>
-      <c r="G5" s="23"/>
-      <c r="H5" s="23"/>
-      <c r="I5" s="23"/>
-      <c r="J5" s="23"/>
-      <c r="K5" s="23"/>
-      <c r="L5" s="23"/>
-      <c r="M5" s="23"/>
-      <c r="N5" s="23"/>
-      <c r="O5" s="23"/>
-      <c r="P5" s="23"/>
-      <c r="Q5" s="23"/>
-      <c r="R5" s="23"/>
-      <c r="S5" s="23"/>
+      <c r="B5" s="24"/>
+      <c r="C5" s="24"/>
+      <c r="D5" s="24"/>
+      <c r="E5" s="24"/>
+      <c r="F5" s="24"/>
+      <c r="G5" s="24"/>
+      <c r="H5" s="24"/>
+      <c r="I5" s="24"/>
+      <c r="J5" s="24"/>
+      <c r="K5" s="24"/>
+      <c r="L5" s="24"/>
+      <c r="M5" s="24"/>
+      <c r="N5" s="24"/>
+      <c r="O5" s="24"/>
+      <c r="P5" s="24"/>
+      <c r="Q5" s="24"/>
+      <c r="R5" s="24"/>
+      <c r="S5" s="24"/>
+      <c r="T5" s="24"/>
     </row>
-    <row r="6" spans="1:19" ht="3" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="7" spans="1:19" s="4" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="13" t="s">
+    <row r="6" spans="1:20" ht="3" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="7" spans="1:20" s="4" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="14" t="s">
         <v>3</v>
       </c>
-      <c r="B7" s="13" t="s">
+      <c r="B7" s="14" t="s">
+        <v>64</v>
+      </c>
+      <c r="C7" s="14" t="s">
         <v>5</v>
       </c>
-      <c r="C7" s="20" t="s">
+      <c r="D7" s="21" t="s">
         <v>10</v>
       </c>
-      <c r="D7" s="13" t="s">
+      <c r="E7" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="E7" s="13" t="s">
+      <c r="F7" s="14" t="s">
         <v>11</v>
       </c>
-      <c r="F7" s="13" t="s">
+      <c r="G7" s="14" t="s">
         <v>6</v>
       </c>
-      <c r="G7" s="13" t="s">
+      <c r="H7" s="14" t="s">
         <v>8</v>
       </c>
-      <c r="H7" s="13" t="s">
+      <c r="I7" s="14" t="s">
         <v>7</v>
       </c>
-      <c r="I7" s="13" t="s">
+      <c r="J7" s="14" t="s">
         <v>20</v>
       </c>
-      <c r="J7" s="13" t="s">
+      <c r="K7" s="14" t="s">
         <v>41</v>
       </c>
-      <c r="K7" s="13" t="s">
+      <c r="L7" s="14" t="s">
         <v>43</v>
       </c>
-      <c r="L7" s="13" t="s">
+      <c r="M7" s="14" t="s">
         <v>44</v>
       </c>
-      <c r="M7" s="14" t="s">
+      <c r="N7" s="15" t="s">
         <v>45</v>
       </c>
-      <c r="N7" s="17" t="s">
+      <c r="O7" s="18" t="s">
         <v>46</v>
       </c>
-      <c r="O7" s="17" t="s">
+      <c r="P7" s="18" t="s">
         <v>47</v>
       </c>
-      <c r="P7" s="15" t="s">
+      <c r="Q7" s="16" t="s">
         <v>60</v>
       </c>
-      <c r="Q7" s="17" t="s">
+      <c r="R7" s="18" t="s">
         <v>55</v>
       </c>
-      <c r="R7" s="17" t="s">
+      <c r="S7" s="18" t="s">
         <v>61</v>
       </c>
-      <c r="S7" s="15" t="s">
+      <c r="T7" s="16" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="8" spans="1:19" s="4" customFormat="1" ht="84" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="14"/>
-      <c r="B8" s="14"/>
-      <c r="C8" s="21"/>
+    <row r="8" spans="1:20" s="4" customFormat="1" ht="84" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="15"/>
+      <c r="B8" s="15"/>
+      <c r="C8" s="15"/>
       <c r="D8" s="22"/>
-      <c r="E8" s="14"/>
-      <c r="F8" s="14"/>
-      <c r="G8" s="14"/>
-      <c r="H8" s="14"/>
-      <c r="I8" s="14"/>
-      <c r="J8" s="14"/>
-      <c r="K8" s="14"/>
-      <c r="L8" s="14"/>
-      <c r="M8" s="19"/>
-      <c r="N8" s="18"/>
-      <c r="O8" s="18"/>
-      <c r="P8" s="16"/>
-      <c r="Q8" s="18"/>
-      <c r="R8" s="18"/>
-      <c r="S8" s="16"/>
+      <c r="E8" s="23"/>
+      <c r="F8" s="15"/>
+      <c r="G8" s="15"/>
+      <c r="H8" s="15"/>
+      <c r="I8" s="15"/>
+      <c r="J8" s="15"/>
+      <c r="K8" s="15"/>
+      <c r="L8" s="15"/>
+      <c r="M8" s="15"/>
+      <c r="N8" s="20"/>
+      <c r="O8" s="19"/>
+      <c r="P8" s="19"/>
+      <c r="Q8" s="17"/>
+      <c r="R8" s="19"/>
+      <c r="S8" s="19"/>
+      <c r="T8" s="17"/>
     </row>
-    <row r="9" spans="1:19" s="9" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:20" s="9" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="B9" s="8" t="s">
+      <c r="B9" s="8"/>
+      <c r="C9" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="C9" s="8" t="s">
+      <c r="D9" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="D9" s="8" t="s">
+      <c r="E9" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="E9" s="8" t="s">
+      <c r="F9" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="F9" s="8" t="s">
+      <c r="G9" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="G9" s="8" t="s">
+      <c r="H9" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="H9" s="8" t="s">
+      <c r="I9" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="I9" s="8" t="s">
+      <c r="J9" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="J9" s="8" t="s">
+      <c r="K9" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="K9" s="8" t="s">
+      <c r="L9" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="L9" s="8" t="s">
+      <c r="M9" s="8" t="s">
         <v>36</v>
       </c>
-      <c r="M9" s="8" t="s">
+      <c r="N9" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="N9" s="8" t="s">
+      <c r="O9" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="O9" s="8" t="s">
+      <c r="P9" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="P9" s="8" t="s">
+      <c r="Q9" s="8" t="s">
         <v>40</v>
       </c>
-      <c r="Q9" s="8" t="s">
+      <c r="R9" s="8" t="s">
         <v>56</v>
       </c>
-      <c r="R9" s="8" t="s">
+      <c r="S9" s="8" t="s">
         <v>57</v>
       </c>
-      <c r="S9" s="8" t="s">
+      <c r="T9" s="8" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="10" spans="1:19" s="4" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:20" s="4" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="B10" s="6" t="s">
+      <c r="B10" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="C10" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="C10" s="7" t="s">
+      <c r="D10" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="D10" s="7" t="s">
+      <c r="E10" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="E10" s="11" t="s">
+      <c r="F10" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="F10" s="7" t="s">
+      <c r="G10" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="G10" s="7" t="s">
+      <c r="H10" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="H10" s="7" t="s">
+      <c r="I10" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="I10" s="7" t="s">
+      <c r="J10" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="J10" s="11" t="s">
+      <c r="K10" s="11" t="s">
         <v>42</v>
       </c>
-      <c r="K10" s="11" t="s">
+      <c r="L10" s="11" t="s">
         <v>51</v>
       </c>
-      <c r="L10" s="11" t="s">
+      <c r="M10" s="11" t="s">
         <v>52</v>
       </c>
-      <c r="M10" s="11" t="s">
+      <c r="N10" s="11" t="s">
         <v>53</v>
       </c>
-      <c r="N10" s="11" t="s">
+      <c r="O10" s="11" t="s">
         <v>54</v>
       </c>
-      <c r="O10" s="25" t="s">
+      <c r="P10" s="13" t="s">
         <v>50</v>
       </c>
-      <c r="P10" s="11" t="s">
+      <c r="Q10" s="11" t="s">
         <v>59</v>
       </c>
-      <c r="Q10" s="12" t="s">
+      <c r="R10" s="12" t="s">
         <v>58</v>
       </c>
-      <c r="R10" s="12" t="s">
+      <c r="S10" s="12" t="s">
         <v>62</v>
       </c>
-      <c r="S10" s="10" t="s">
+      <c r="T10" s="10" t="s">
         <v>24</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="25">
-    <mergeCell ref="F2:S2"/>
-    <mergeCell ref="F3:S3"/>
-    <mergeCell ref="A4:S4"/>
-    <mergeCell ref="A5:S5"/>
-    <mergeCell ref="A2:D2"/>
-    <mergeCell ref="A3:D3"/>
+  <mergeCells count="26">
+    <mergeCell ref="G2:T2"/>
+    <mergeCell ref="G3:T3"/>
+    <mergeCell ref="A4:T4"/>
+    <mergeCell ref="A5:T5"/>
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A3:E3"/>
     <mergeCell ref="A7:A8"/>
-    <mergeCell ref="B7:B8"/>
     <mergeCell ref="C7:C8"/>
     <mergeCell ref="D7:D8"/>
-    <mergeCell ref="H7:H8"/>
     <mergeCell ref="E7:E8"/>
+    <mergeCell ref="I7:I8"/>
     <mergeCell ref="F7:F8"/>
     <mergeCell ref="G7:G8"/>
-    <mergeCell ref="I7:I8"/>
+    <mergeCell ref="H7:H8"/>
+    <mergeCell ref="B7:B8"/>
+    <mergeCell ref="J7:J8"/>
+    <mergeCell ref="T7:T8"/>
     <mergeCell ref="S7:S8"/>
-    <mergeCell ref="R7:R8"/>
-    <mergeCell ref="J7:J8"/>
+    <mergeCell ref="K7:K8"/>
+    <mergeCell ref="M7:M8"/>
+    <mergeCell ref="N7:N8"/>
     <mergeCell ref="L7:L8"/>
-    <mergeCell ref="M7:M8"/>
-    <mergeCell ref="K7:K8"/>
-    <mergeCell ref="N7:N8"/>
     <mergeCell ref="O7:O8"/>
     <mergeCell ref="P7:P8"/>
     <mergeCell ref="Q7:Q8"/>
+    <mergeCell ref="R7:R8"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.6" right="0.5" top="0.6" bottom="0.5" header="0.05" footer="0.05"/>

</xml_diff>